<commit_message>
Respaldo independiente: 2026-03-16 16:41
</commit_message>
<xml_diff>
--- a/DatosLab1.xlsx
+++ b/DatosLab1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="133">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -287,6 +287,129 @@
   </si>
   <si>
     <t>52kg</t>
+  </si>
+  <si>
+    <t>mariafernandalopez@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Maria Fernanda Lopez Lopez</t>
+  </si>
+  <si>
+    <t>jdanielleon@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan Daniel León Lozano </t>
+  </si>
+  <si>
+    <t>165 cm</t>
+  </si>
+  <si>
+    <t>rmontilla@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raquel Alicia Montilla Pérez </t>
+  </si>
+  <si>
+    <t xml:space="preserve">157.2 cm </t>
+  </si>
+  <si>
+    <t>74.3 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82.9 cm </t>
+  </si>
+  <si>
+    <t>mauricioadiaz@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Mauricio Andres Diaz Falco</t>
+  </si>
+  <si>
+    <t>miguelasanchez@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Miguel Ángel Sánchez Mercado</t>
+  </si>
+  <si>
+    <t>anunezd@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amalfi Nuñez Doria </t>
+  </si>
+  <si>
+    <t>jsguerra@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Juan Sebastian Guerra Rojas</t>
+  </si>
+  <si>
+    <t>cparedesd@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carla Paredes Díaz </t>
+  </si>
+  <si>
+    <t>xmaussa@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Xhiara Elena Maussa Oviedo</t>
+  </si>
+  <si>
+    <t>nulo</t>
+  </si>
+  <si>
+    <t>marioamartinez@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mario Andres Martinez Lagares </t>
+  </si>
+  <si>
+    <t>yinunez@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Yeison Isaac nuñez garavito</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>lestivenregino@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Luis Estiven Regino De La Rosa</t>
+  </si>
+  <si>
+    <t>mariaangelicagonzalez@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>María Angelica González Peralta</t>
+  </si>
+  <si>
+    <t>vcausill@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Verónica Causil Lozano</t>
+  </si>
+  <si>
+    <t>mmedranoc@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t>Matías Medrano Causil</t>
+  </si>
+  <si>
+    <t>310 8335746</t>
+  </si>
+  <si>
+    <t>ajosepramos@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angel Josep Ramos Paez </t>
+  </si>
+  <si>
+    <t>mamorales@correo.unicordoba.edu.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mario Alfonso Morales Rivera </t>
   </si>
 </sst>
 </file>
@@ -323,12 +446,21 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="14" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -418,7 +550,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Y21" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:Y38" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="25">
     <tableColumn name="Marca temporal" id="1"/>
     <tableColumn name="Dirección de correo electrónico" id="2"/>
@@ -2291,6 +2423,1315 @@
         <v>34.0</v>
       </c>
     </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="5">
+        <v>46096.41745462963</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="6">
+        <v>1.063147052E9</v>
+      </c>
+      <c r="E22" s="7">
+        <v>39015.0</v>
+      </c>
+      <c r="F22" s="6">
+        <v>19.0</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="6">
+        <v>3.044415554E9</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M22" s="6">
+        <v>95.0</v>
+      </c>
+      <c r="N22" s="6">
+        <v>94.0</v>
+      </c>
+      <c r="O22" s="6">
+        <v>69.0</v>
+      </c>
+      <c r="P22" s="6">
+        <v>156.5</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>41.2</v>
+      </c>
+      <c r="R22" s="6">
+        <v>56.4</v>
+      </c>
+      <c r="S22" s="6">
+        <v>16.8</v>
+      </c>
+      <c r="T22" s="6">
+        <v>25.2</v>
+      </c>
+      <c r="U22" s="6">
+        <v>29.2</v>
+      </c>
+      <c r="V22" s="6">
+        <v>1.6</v>
+      </c>
+      <c r="W22" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X22" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="Y22" s="6">
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="5">
+        <v>46096.43165481482</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1.0428251199E10</v>
+      </c>
+      <c r="E23" s="7">
+        <v>39608.0</v>
+      </c>
+      <c r="F23" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H23" s="6">
+        <v>3.207702762E9</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M23" s="6">
+        <v>80.0</v>
+      </c>
+      <c r="N23" s="6">
+        <v>128.0</v>
+      </c>
+      <c r="O23" s="6">
+        <v>70.0</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>1.8</v>
+      </c>
+      <c r="R23" s="6">
+        <v>71.5</v>
+      </c>
+      <c r="S23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="T23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="U23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="V23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="W23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="X23" s="6">
+        <v>28.0</v>
+      </c>
+      <c r="Y23" s="6">
+        <v>38.0</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="5">
+        <v>46096.43492329861</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D24" s="6">
+        <v>5841206.0</v>
+      </c>
+      <c r="E24" s="7">
+        <v>39344.0</v>
+      </c>
+      <c r="F24" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" s="6">
+        <v>3.046347212E9</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M24" s="6">
+        <v>92.0</v>
+      </c>
+      <c r="N24" s="6">
+        <v>125.0</v>
+      </c>
+      <c r="O24" s="6">
+        <v>78.0</v>
+      </c>
+      <c r="P24" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q24" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R24" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="S24" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="T24" s="6">
+        <v>40.0</v>
+      </c>
+      <c r="U24" s="6">
+        <v>42.3</v>
+      </c>
+      <c r="V24" s="6">
+        <v>2.3</v>
+      </c>
+      <c r="W24" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="X24" s="6">
+        <v>28.0</v>
+      </c>
+      <c r="Y24" s="6">
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="5">
+        <v>46096.440802627316</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D25" s="6">
+        <v>1.068418499E9</v>
+      </c>
+      <c r="E25" s="7">
+        <v>38966.0</v>
+      </c>
+      <c r="F25" s="6">
+        <v>19.0</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H25" s="6">
+        <v>3.126184367E9</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M25" s="6">
+        <v>71.0</v>
+      </c>
+      <c r="N25" s="6">
+        <v>129.0</v>
+      </c>
+      <c r="O25" s="6">
+        <v>66.0</v>
+      </c>
+      <c r="P25" s="6">
+        <v>181.0</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>62.6</v>
+      </c>
+      <c r="R25" s="6">
+        <v>69.6</v>
+      </c>
+      <c r="S25" s="6">
+        <v>19.3</v>
+      </c>
+      <c r="T25" s="6">
+        <v>10.4</v>
+      </c>
+      <c r="U25" s="6">
+        <v>53.3</v>
+      </c>
+      <c r="V25" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="W25" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X25" s="6">
+        <v>46.0</v>
+      </c>
+      <c r="Y25" s="6">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="5">
+        <v>46096.446570162036</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1.068417696E9</v>
+      </c>
+      <c r="E26" s="7">
+        <v>38541.0</v>
+      </c>
+      <c r="F26" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H26" s="6">
+        <v>3.005050726E9</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L26" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M26" s="6">
+        <v>73.0</v>
+      </c>
+      <c r="N26" s="6">
+        <v>127.0</v>
+      </c>
+      <c r="O26" s="6">
+        <v>76.0</v>
+      </c>
+      <c r="P26" s="6">
+        <v>189.5</v>
+      </c>
+      <c r="Q26" s="6">
+        <v>97.0</v>
+      </c>
+      <c r="R26" s="6">
+        <v>88.6</v>
+      </c>
+      <c r="S26" s="6">
+        <v>27.0</v>
+      </c>
+      <c r="T26" s="6">
+        <v>23.3</v>
+      </c>
+      <c r="U26" s="6">
+        <v>70.7</v>
+      </c>
+      <c r="V26" s="6">
+        <v>3.7</v>
+      </c>
+      <c r="W26" s="6">
+        <v>5.5</v>
+      </c>
+      <c r="X26" s="6">
+        <v>54.0</v>
+      </c>
+      <c r="Y26" s="6">
+        <v>46.0</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="5">
+        <v>46096.44907645833</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" s="6">
+        <v>1.063721761E9</v>
+      </c>
+      <c r="E27" s="7">
+        <v>39084.0</v>
+      </c>
+      <c r="F27" s="6">
+        <v>19.0</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H27" s="6">
+        <v>3.237357969E9</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M27" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="N27" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="O27" s="6">
+        <v>72.0</v>
+      </c>
+      <c r="P27" s="6">
+        <v>1.57</v>
+      </c>
+      <c r="Q27" s="6">
+        <v>49.2</v>
+      </c>
+      <c r="R27" s="6">
+        <v>67.4</v>
+      </c>
+      <c r="S27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T27" s="6">
+        <v>28.5</v>
+      </c>
+      <c r="U27" s="6">
+        <v>33.3</v>
+      </c>
+      <c r="V27" s="6">
+        <v>1.8</v>
+      </c>
+      <c r="W27" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X27" s="6">
+        <v>22.0</v>
+      </c>
+      <c r="Y27" s="6">
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="5">
+        <v>46096.45084417824</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="6">
+        <v>1.067897721E9</v>
+      </c>
+      <c r="E28" s="7">
+        <v>39060.0</v>
+      </c>
+      <c r="F28" s="6">
+        <v>19.0</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H28" s="6">
+        <v>3.128883197E9</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M28" s="6">
+        <v>117.0</v>
+      </c>
+      <c r="N28" s="6">
+        <v>162.0</v>
+      </c>
+      <c r="O28" s="6">
+        <v>102.0</v>
+      </c>
+      <c r="P28" s="6">
+        <v>167.5</v>
+      </c>
+      <c r="Q28" s="6">
+        <v>94.0</v>
+      </c>
+      <c r="R28" s="6">
+        <v>92.8</v>
+      </c>
+      <c r="S28" s="6">
+        <v>33.5</v>
+      </c>
+      <c r="T28" s="6">
+        <v>32.8</v>
+      </c>
+      <c r="U28" s="6">
+        <v>60.0</v>
+      </c>
+      <c r="V28" s="6">
+        <v>3.2</v>
+      </c>
+      <c r="W28" s="6">
+        <v>11.5</v>
+      </c>
+      <c r="X28" s="6">
+        <v>24.0</v>
+      </c>
+      <c r="Y28" s="6">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="5">
+        <v>46096.53411305556</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" s="6">
+        <v>1.067872099E9</v>
+      </c>
+      <c r="E29" s="7">
+        <v>39188.0</v>
+      </c>
+      <c r="F29" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" s="6">
+        <v>3.205702281E9</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K29" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L29" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M29" s="6">
+        <v>86.0</v>
+      </c>
+      <c r="N29" s="6">
+        <v>106.0</v>
+      </c>
+      <c r="O29" s="6">
+        <v>84.0</v>
+      </c>
+      <c r="P29" s="6">
+        <v>158.4</v>
+      </c>
+      <c r="Q29" s="6">
+        <v>49.0</v>
+      </c>
+      <c r="R29" s="6">
+        <v>66.4</v>
+      </c>
+      <c r="S29" s="6">
+        <v>19.5</v>
+      </c>
+      <c r="T29" s="6">
+        <v>28.2</v>
+      </c>
+      <c r="U29" s="6">
+        <v>33.4</v>
+      </c>
+      <c r="V29" s="6">
+        <v>1.3</v>
+      </c>
+      <c r="W29" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="Y29" s="6">
+        <v>22.0</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="5">
+        <v>46096.5357474537</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D30" s="6">
+        <v>1.137978448E9</v>
+      </c>
+      <c r="E30" s="7">
+        <v>39577.0</v>
+      </c>
+      <c r="F30" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30" s="6">
+        <v>3.187389644E9</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L30" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M30" s="6">
+        <v>82.0</v>
+      </c>
+      <c r="N30" s="6">
+        <v>116.0</v>
+      </c>
+      <c r="O30" s="6">
+        <v>67.0</v>
+      </c>
+      <c r="P30" s="6">
+        <v>165.5</v>
+      </c>
+      <c r="Q30" s="6">
+        <v>51.7</v>
+      </c>
+      <c r="R30" s="6">
+        <v>65.6</v>
+      </c>
+      <c r="S30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="T30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="U30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="V30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="W30" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="X30" s="6">
+        <v>26.0</v>
+      </c>
+      <c r="Y30" s="6">
+        <v>24.0</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="5">
+        <v>46096.57047515047</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="6">
+        <v>1.067858453E9</v>
+      </c>
+      <c r="E31" s="7">
+        <v>38647.0</v>
+      </c>
+      <c r="F31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H31" s="6">
+        <v>3.137965692E9</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M31" s="6">
+        <v>88.0</v>
+      </c>
+      <c r="N31" s="6">
+        <v>93.0</v>
+      </c>
+      <c r="O31" s="6">
+        <v>56.0</v>
+      </c>
+      <c r="P31" s="6">
+        <v>171.5</v>
+      </c>
+      <c r="Q31" s="6">
+        <v>51.5</v>
+      </c>
+      <c r="R31" s="6">
+        <v>65.0</v>
+      </c>
+      <c r="S31" s="6">
+        <v>17.5</v>
+      </c>
+      <c r="T31" s="6">
+        <v>11.6</v>
+      </c>
+      <c r="U31" s="6">
+        <v>43.2</v>
+      </c>
+      <c r="V31" s="6">
+        <v>2.3</v>
+      </c>
+      <c r="W31" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X31" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="Y31" s="6">
+        <v>40.0</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="5">
+        <v>46096.57906510417</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D32" s="6">
+        <v>1.03181472E9</v>
+      </c>
+      <c r="E32" s="7">
+        <v>39639.0</v>
+      </c>
+      <c r="F32" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H32" s="6">
+        <v>3.011483166E9</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M32" s="6">
+        <v>95.0</v>
+      </c>
+      <c r="N32" s="6">
+        <v>132.0</v>
+      </c>
+      <c r="O32" s="6">
+        <v>67.0</v>
+      </c>
+      <c r="P32" s="6">
+        <v>172.5</v>
+      </c>
+      <c r="Q32" s="6">
+        <v>60.6</v>
+      </c>
+      <c r="R32" s="6">
+        <v>75.5</v>
+      </c>
+      <c r="S32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="T32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="U32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="V32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="W32" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="X32" s="6">
+        <v>46.0</v>
+      </c>
+      <c r="Y32" s="6">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="5">
+        <v>46096.583023935185</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D33" s="6">
+        <v>1.062964598E9</v>
+      </c>
+      <c r="E33" s="7">
+        <v>39456.0</v>
+      </c>
+      <c r="F33" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H33" s="6">
+        <v>3.207879806E9</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M33" s="6">
+        <v>56.0</v>
+      </c>
+      <c r="N33" s="6">
+        <v>122.0</v>
+      </c>
+      <c r="O33" s="6">
+        <v>84.0</v>
+      </c>
+      <c r="P33" s="6">
+        <v>164.7</v>
+      </c>
+      <c r="Q33" s="6">
+        <v>50.3</v>
+      </c>
+      <c r="R33" s="6">
+        <v>686.0</v>
+      </c>
+      <c r="S33" s="6">
+        <v>18.5</v>
+      </c>
+      <c r="T33" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="U33" s="6">
+        <v>42.5</v>
+      </c>
+      <c r="V33" s="6">
+        <v>2.3</v>
+      </c>
+      <c r="W33" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X33" s="6">
+        <v>26.0</v>
+      </c>
+      <c r="Y33" s="6">
+        <v>22.0</v>
+      </c>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="5">
+        <v>46096.592872546295</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D34" s="6">
+        <v>1.06243477E9</v>
+      </c>
+      <c r="E34" s="7">
+        <v>39204.0</v>
+      </c>
+      <c r="F34" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H34" s="6">
+        <v>3.001126316E9</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M34" s="6">
+        <v>87.0</v>
+      </c>
+      <c r="N34" s="6">
+        <v>105.0</v>
+      </c>
+      <c r="O34" s="6">
+        <v>75.0</v>
+      </c>
+      <c r="P34" s="6">
+        <v>160.8</v>
+      </c>
+      <c r="Q34" s="6">
+        <v>47.6</v>
+      </c>
+      <c r="R34" s="6">
+        <v>60.5</v>
+      </c>
+      <c r="S34" s="6">
+        <v>18.4</v>
+      </c>
+      <c r="T34" s="6">
+        <v>23.8</v>
+      </c>
+      <c r="U34" s="6">
+        <v>34.4</v>
+      </c>
+      <c r="V34" s="6">
+        <v>1.9</v>
+      </c>
+      <c r="W34" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X34" s="6">
+        <v>26.0</v>
+      </c>
+      <c r="Y34" s="6">
+        <v>22.0</v>
+      </c>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="5">
+        <v>46096.66357421296</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="6">
+        <v>1.063285784E9</v>
+      </c>
+      <c r="E35" s="7">
+        <v>39451.0</v>
+      </c>
+      <c r="F35" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H35" s="6">
+        <v>3.225022182E9</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M35" s="6">
+        <v>92.0</v>
+      </c>
+      <c r="N35" s="6">
+        <v>125.0</v>
+      </c>
+      <c r="O35" s="6">
+        <v>74.0</v>
+      </c>
+      <c r="P35" s="6">
+        <v>160.0</v>
+      </c>
+      <c r="Q35" s="6">
+        <v>63.7</v>
+      </c>
+      <c r="R35" s="6">
+        <v>71.0</v>
+      </c>
+      <c r="S35" s="6">
+        <v>24.9</v>
+      </c>
+      <c r="T35" s="6">
+        <v>37.5</v>
+      </c>
+      <c r="U35" s="6">
+        <v>37.8</v>
+      </c>
+      <c r="V35" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="W35" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="X35" s="6">
+        <v>28.0</v>
+      </c>
+      <c r="Y35" s="6">
+        <v>32.0</v>
+      </c>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="5">
+        <v>46096.675264618054</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D36" s="6">
+        <v>1.067878777E9</v>
+      </c>
+      <c r="E36" s="7">
+        <v>39259.0</v>
+      </c>
+      <c r="F36" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M36" s="6">
+        <v>79.0</v>
+      </c>
+      <c r="N36" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="O36" s="6">
+        <v>81.0</v>
+      </c>
+      <c r="P36" s="6">
+        <v>178.4</v>
+      </c>
+      <c r="Q36" s="6">
+        <v>60.6</v>
+      </c>
+      <c r="R36" s="6">
+        <v>70.0</v>
+      </c>
+      <c r="S36" s="6">
+        <v>19.0</v>
+      </c>
+      <c r="T36" s="6">
+        <v>14.9</v>
+      </c>
+      <c r="U36" s="6">
+        <v>49.0</v>
+      </c>
+      <c r="V36" s="6">
+        <v>2.6</v>
+      </c>
+      <c r="W36" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="X36" s="6">
+        <v>30.0</v>
+      </c>
+      <c r="Y36" s="6">
+        <v>34.0</v>
+      </c>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="5">
+        <v>46096.73550708333</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D37" s="6">
+        <v>1.067164119E9</v>
+      </c>
+      <c r="E37" s="7">
+        <v>39427.0</v>
+      </c>
+      <c r="F37" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H37" s="6">
+        <v>3.005295556E9</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M37" s="6">
+        <v>76.0</v>
+      </c>
+      <c r="N37" s="6">
+        <v>143.0</v>
+      </c>
+      <c r="O37" s="6">
+        <v>78.0</v>
+      </c>
+      <c r="P37" s="6">
+        <v>1.72</v>
+      </c>
+      <c r="Q37" s="6">
+        <v>74.0</v>
+      </c>
+      <c r="R37" s="6">
+        <v>72.0</v>
+      </c>
+      <c r="S37" s="6">
+        <v>253.1</v>
+      </c>
+      <c r="T37" s="6">
+        <v>16.5</v>
+      </c>
+      <c r="U37" s="6">
+        <v>59.6</v>
+      </c>
+      <c r="V37" s="6">
+        <v>3.1</v>
+      </c>
+      <c r="W37" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="X37" s="6">
+        <v>50.0</v>
+      </c>
+      <c r="Y37" s="6">
+        <v>52.0</v>
+      </c>
+    </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="5">
+        <v>46097.4040125</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D38" s="6">
+        <v>7.8689764E7</v>
+      </c>
+      <c r="E38" s="7">
+        <v>24092.0</v>
+      </c>
+      <c r="F38" s="6">
+        <v>60.0</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H38" s="6">
+        <v>3.17450707E9</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="L38" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="M38" s="6">
+        <v>59.0</v>
+      </c>
+      <c r="N38" s="6">
+        <v>142.0</v>
+      </c>
+      <c r="O38" s="6">
+        <v>85.0</v>
+      </c>
+      <c r="P38" s="6">
+        <v>163.9</v>
+      </c>
+      <c r="Q38" s="6">
+        <v>71.3</v>
+      </c>
+      <c r="R38" s="6">
+        <v>86.7</v>
+      </c>
+      <c r="S38" s="6">
+        <v>26.5</v>
+      </c>
+      <c r="T38" s="6">
+        <v>26.5</v>
+      </c>
+      <c r="U38" s="6">
+        <v>49.8</v>
+      </c>
+      <c r="V38" s="6">
+        <v>2.7</v>
+      </c>
+      <c r="W38" s="6">
+        <v>13.0</v>
+      </c>
+      <c r="X38" s="6">
+        <v>42.0</v>
+      </c>
+      <c r="Y38" s="6">
+        <v>40.0</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>